<commit_message>
Add scraping 15-04-2026 data + updated master
- New CSV: anas_obras_20260415_125514.csv (50 obras, 48 after dedup)
- Master updated with Avanz_15-04-2026_1256 column
- 675 values updated, 525 preserved from enrichment

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/master_avanzamento.xlsx
+++ b/data/processed/master_avanzamento.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD49"/>
+  <dimension ref="A1:AE49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,6 +564,11 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>Avanz_15-04-2026_1256</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>Differenza</t>
         </is>
       </c>
@@ -712,6 +717,11 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
+          <t>2,70</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -860,6 +870,11 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
+          <t>83,14</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1008,6 +1023,11 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
+          <t>1,08</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1156,6 +1176,11 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
+          <t>39,57</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1304,6 +1329,11 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
+          <t>79,71</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1452,6 +1482,11 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
+          <t>10,65</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1600,6 +1635,11 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
+          <t>11,95</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1748,6 +1788,11 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
+          <t>95,17</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1896,6 +1941,11 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
+          <t>50,80</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2040,6 +2090,11 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
+          <t>2,52</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2188,6 +2243,11 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
+          <t>25,13</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2336,6 +2396,11 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
+          <t>92,33</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2480,6 +2545,11 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
+          <t>14,90</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2624,6 +2694,11 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
+          <t>3,09</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2768,6 +2843,11 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
+          <t>18,87</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2912,6 +2992,11 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
+          <t>38,05</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3056,6 +3141,11 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
+          <t>3,22</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3200,6 +3290,11 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
+          <t>29,87</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3348,6 +3443,11 @@
       </c>
       <c r="AD20" t="inlineStr">
         <is>
+          <t>78,03</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3496,6 +3596,11 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
+          <t>98,31</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3640,6 +3745,11 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
+          <t>99,77</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3788,6 +3898,11 @@
       </c>
       <c r="AD23" t="inlineStr">
         <is>
+          <t>92,07</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3936,6 +4051,11 @@
       </c>
       <c r="AD24" t="inlineStr">
         <is>
+          <t>96,08</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4084,6 +4204,11 @@
       </c>
       <c r="AD25" t="inlineStr">
         <is>
+          <t>99,94</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4232,6 +4357,11 @@
       </c>
       <c r="AD26" t="inlineStr">
         <is>
+          <t>19,13</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4380,6 +4510,11 @@
       </c>
       <c r="AD27" t="inlineStr">
         <is>
+          <t>7,27</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4528,6 +4663,11 @@
       </c>
       <c r="AD28" t="inlineStr">
         <is>
+          <t>41,84</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4676,6 +4816,11 @@
       </c>
       <c r="AD29" t="inlineStr">
         <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4824,6 +4969,11 @@
       </c>
       <c r="AD30" t="inlineStr">
         <is>
+          <t>89,19</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4972,6 +5122,11 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
+          <t>98,88</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5120,6 +5275,11 @@
       </c>
       <c r="AD32" t="inlineStr">
         <is>
+          <t>58,95</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5268,6 +5428,11 @@
       </c>
       <c r="AD33" t="inlineStr">
         <is>
+          <t>60,58</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5416,6 +5581,11 @@
       </c>
       <c r="AD34" t="inlineStr">
         <is>
+          <t>45,70</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5564,6 +5734,11 @@
       </c>
       <c r="AD35" t="inlineStr">
         <is>
+          <t>23,77</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5712,6 +5887,11 @@
       </c>
       <c r="AD36" t="inlineStr">
         <is>
+          <t>37,11</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5860,6 +6040,11 @@
       </c>
       <c r="AD37" t="inlineStr">
         <is>
+          <t>67,58</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6004,6 +6189,11 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
+          <t>1,20</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6148,6 +6338,11 @@
       </c>
       <c r="AD39" t="inlineStr">
         <is>
+          <t>0,98</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6292,6 +6487,11 @@
       </c>
       <c r="AD40" t="inlineStr">
         <is>
+          <t>0,97</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6436,6 +6636,11 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
+          <t>1,02</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6580,6 +6785,11 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
+          <t>1,48</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6728,6 +6938,11 @@
       </c>
       <c r="AD43" t="inlineStr">
         <is>
+          <t>95,52</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6876,6 +7091,11 @@
       </c>
       <c r="AD44" t="inlineStr">
         <is>
+          <t>17,86</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7024,6 +7244,11 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
+          <t>79,69</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7172,6 +7397,11 @@
       </c>
       <c r="AD46" t="inlineStr">
         <is>
+          <t>1,33</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7320,6 +7550,11 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
+          <t>87,98</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7468,6 +7703,11 @@
       </c>
       <c r="AD48" t="inlineStr">
         <is>
+          <t>10,69</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7615,6 +7855,11 @@
         </is>
       </c>
       <c r="AD49" t="inlineStr">
+        <is>
+          <t>87,25</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>

</xml_diff>

<commit_message>
Update master state — 2026-05-04 10:31
6 file sincronizzati dalla UI PAVIMOD:
  - data/processed/master_avanzamento.xlsx
  - data/cache/opencup_cache.json
  - data/processed/anas_obras_20260411_190348.csv
  - data/processed/anas_obras_20260411_190949.csv
  - data/processed/anas_obras_20260411_191350.csv
  - data/processed/anas_obras_20260415_125514.csv
</commit_message>
<xml_diff>
--- a/data/processed/master_avanzamento.xlsx
+++ b/data/processed/master_avanzamento.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE49"/>
+  <dimension ref="A1:AF49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,6 +569,11 @@
       </c>
       <c r="AE1" t="inlineStr">
         <is>
+          <t>Avanz_04-05-2026_1025</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
           <t>Differenza</t>
         </is>
       </c>
@@ -722,6 +727,11 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
+          <t>2,70</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -875,6 +885,11 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
+          <t>83,14</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1028,6 +1043,11 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
+          <t>1,08</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1181,6 +1201,11 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
+          <t>39,57</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1334,6 +1359,11 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
+          <t>79,71</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1487,6 +1517,11 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
+          <t>10,65</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1640,6 +1675,11 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
+          <t>11,95</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1793,6 +1833,11 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
+          <t>95,17</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -1946,6 +1991,11 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
+          <t>50,80</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2095,6 +2145,11 @@
       </c>
       <c r="AE11" t="inlineStr">
         <is>
+          <t>2,52</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2248,6 +2303,11 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
+          <t>25,13</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2401,6 +2461,11 @@
       </c>
       <c r="AE13" t="inlineStr">
         <is>
+          <t>92,33</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2550,6 +2615,11 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
+          <t>14,90</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2699,6 +2769,11 @@
       </c>
       <c r="AE15" t="inlineStr">
         <is>
+          <t>3,09</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2848,6 +2923,11 @@
       </c>
       <c r="AE16" t="inlineStr">
         <is>
+          <t>18,87</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -2997,6 +3077,11 @@
       </c>
       <c r="AE17" t="inlineStr">
         <is>
+          <t>38,05</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3146,6 +3231,11 @@
       </c>
       <c r="AE18" t="inlineStr">
         <is>
+          <t>3,22</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3295,6 +3385,11 @@
       </c>
       <c r="AE19" t="inlineStr">
         <is>
+          <t>29,87</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3448,6 +3543,11 @@
       </c>
       <c r="AE20" t="inlineStr">
         <is>
+          <t>78,03</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3601,6 +3701,11 @@
       </c>
       <c r="AE21" t="inlineStr">
         <is>
+          <t>98,31</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3750,6 +3855,11 @@
       </c>
       <c r="AE22" t="inlineStr">
         <is>
+          <t>99,77</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3903,6 +4013,11 @@
       </c>
       <c r="AE23" t="inlineStr">
         <is>
+          <t>92,07</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4056,6 +4171,11 @@
       </c>
       <c r="AE24" t="inlineStr">
         <is>
+          <t>96,08</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4209,6 +4329,11 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
+          <t>99,94</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4362,6 +4487,11 @@
       </c>
       <c r="AE26" t="inlineStr">
         <is>
+          <t>19,13</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4515,6 +4645,11 @@
       </c>
       <c r="AE27" t="inlineStr">
         <is>
+          <t>7,27</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4668,6 +4803,11 @@
       </c>
       <c r="AE28" t="inlineStr">
         <is>
+          <t>41,84</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4821,6 +4961,11 @@
       </c>
       <c r="AE29" t="inlineStr">
         <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4974,6 +5119,11 @@
       </c>
       <c r="AE30" t="inlineStr">
         <is>
+          <t>89,19</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5127,6 +5277,11 @@
       </c>
       <c r="AE31" t="inlineStr">
         <is>
+          <t>98,88</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5280,6 +5435,11 @@
       </c>
       <c r="AE32" t="inlineStr">
         <is>
+          <t>58,95</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5433,6 +5593,11 @@
       </c>
       <c r="AE33" t="inlineStr">
         <is>
+          <t>60,58</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5586,6 +5751,11 @@
       </c>
       <c r="AE34" t="inlineStr">
         <is>
+          <t>45,70</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5739,6 +5909,11 @@
       </c>
       <c r="AE35" t="inlineStr">
         <is>
+          <t>23,77</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5892,6 +6067,11 @@
       </c>
       <c r="AE36" t="inlineStr">
         <is>
+          <t>37,11</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6045,6 +6225,11 @@
       </c>
       <c r="AE37" t="inlineStr">
         <is>
+          <t>67,58</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6194,6 +6379,11 @@
       </c>
       <c r="AE38" t="inlineStr">
         <is>
+          <t>1,20</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6343,6 +6533,11 @@
       </c>
       <c r="AE39" t="inlineStr">
         <is>
+          <t>0,98</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6492,6 +6687,11 @@
       </c>
       <c r="AE40" t="inlineStr">
         <is>
+          <t>0,97</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6641,6 +6841,11 @@
       </c>
       <c r="AE41" t="inlineStr">
         <is>
+          <t>1,02</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6790,6 +6995,11 @@
       </c>
       <c r="AE42" t="inlineStr">
         <is>
+          <t>1,48</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -6943,6 +7153,11 @@
       </c>
       <c r="AE43" t="inlineStr">
         <is>
+          <t>95,52</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7096,6 +7311,11 @@
       </c>
       <c r="AE44" t="inlineStr">
         <is>
+          <t>17,86</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7249,6 +7469,11 @@
       </c>
       <c r="AE45" t="inlineStr">
         <is>
+          <t>79,69</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7402,6 +7627,11 @@
       </c>
       <c r="AE46" t="inlineStr">
         <is>
+          <t>1,33</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7555,6 +7785,11 @@
       </c>
       <c r="AE47" t="inlineStr">
         <is>
+          <t>87,98</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7708,6 +7943,11 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
+          <t>10,69</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -7860,6 +8100,11 @@
         </is>
       </c>
       <c r="AE49" t="inlineStr">
+        <is>
+          <t>87,25</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>

</xml_diff>

<commit_message>
Fix silent stale-CSV fallback + publish real June master
app.py (_hilo_scraper): use the CSV that scrape() actually returns instead
of ultimo_csv() (newest file on disk). When the scrape gets no data from
ANAS (e.g. the server's IP is blocked/timed out by stradeanas.it), scrape()
returns csv=None; previously the thread fell back to the newest OLD CSV and
built an Avanz_ column from stale data, showing a fake 0% Differenza. Now it
surfaces a clear error and skips the comparativo so the master is not
overwritten with old values.

master_avanzamento.xlsx: rebuilt from a host that can reach ANAS, adding the
real Avanz_16-06-2026 column (42/49 works moved vs May) so the deployed app
shows current data. Render's datacenter IP cannot scrape ANAS directly.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/master_avanzamento.xlsx
+++ b/data/processed/master_avanzamento.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF49"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -574,6 +574,16 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>Avanz_16-06-2026_1136</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>VTiger</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>Differenza</t>
         </is>
       </c>
@@ -732,7 +742,13 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>3,53</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>+0.8%</t>
         </is>
       </c>
     </row>
@@ -890,7 +906,13 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>84,38</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>+1.2%</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1070,13 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1,87</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>+0.8%</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1234,13 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>44,24</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>+4.7%</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1398,13 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>83,00</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>+3.3%</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1562,13 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>12,92</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>+2.3%</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1726,13 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16,63</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>+4.7%</t>
         </is>
       </c>
     </row>
@@ -1836,9 +1888,11 @@
           <t>95,17</t>
         </is>
       </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Obra Conclusa (probable)</t>
         </is>
       </c>
     </row>
@@ -1996,7 +2050,13 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>58,74</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>+7.9%</t>
         </is>
       </c>
     </row>
@@ -2053,10 +2113,14 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>03-04-2025</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>07-05-2026</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2028-02-07</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>84.720</t>
@@ -2150,7 +2214,13 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>3,12</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>+0.6%</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2378,13 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27,49</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>+2.4%</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2446,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2025-10-22</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2465,6 +2541,12 @@
         </is>
       </c>
       <c r="AF13" t="inlineStr">
+        <is>
+          <t>92,33</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
@@ -2620,7 +2702,13 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18,51</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>+3.6%</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2862,13 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>5,67</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>+2.6%</t>
         </is>
       </c>
     </row>
@@ -2928,7 +3022,13 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>21,15</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>+2.3%</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3182,13 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>42,02</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>+4.0%</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3250,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2028-07-31</t>
+          <t>2028-12-31</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -3236,6 +3342,12 @@
       </c>
       <c r="AF18" t="inlineStr">
         <is>
+          <t>3,22</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -3298,7 +3410,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -3390,7 +3502,13 @@
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33,87</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>+4.0%</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3666,13 @@
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>87,37</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>+9.3%</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3830,13 @@
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>99,06</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>+0.8%</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3990,13 @@
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>99,92</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4154,13 @@
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>92,47</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>+0.4%</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4318,13 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>96,42</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>+0.3%</t>
         </is>
       </c>
     </row>
@@ -4334,6 +4482,12 @@
       </c>
       <c r="AF25" t="inlineStr">
         <is>
+          <t>99,94</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -4492,7 +4646,13 @@
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>24,48</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>+5.4%</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4810,13 @@
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>7,29</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4974,13 @@
       </c>
       <c r="AF28" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>46,31</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>+4.5%</t>
         </is>
       </c>
     </row>
@@ -4966,6 +5138,12 @@
       </c>
       <c r="AF29" t="inlineStr">
         <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr">
+        <is>
           <t>0%</t>
         </is>
       </c>
@@ -5124,7 +5302,13 @@
       </c>
       <c r="AF30" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>92,15</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>+3.0%</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5370,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -5281,6 +5465,12 @@
         </is>
       </c>
       <c r="AF31" t="inlineStr">
+        <is>
+          <t>98,88</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
@@ -5344,7 +5534,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -5439,6 +5629,12 @@
         </is>
       </c>
       <c r="AF32" t="inlineStr">
+        <is>
+          <t>58,95</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
@@ -5598,7 +5794,13 @@
       </c>
       <c r="AF33" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>62,65</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>+2.1%</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5958,13 @@
       </c>
       <c r="AF34" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>49,15</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>+3.4%</t>
         </is>
       </c>
     </row>
@@ -5914,7 +6122,13 @@
       </c>
       <c r="AF35" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>26,23</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>+2.5%</t>
         </is>
       </c>
     </row>
@@ -5956,7 +6170,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>VALORI S.C.A R.L.</t>
+          <t>VALORI S.C.A R.L. - CONSORZIO STABI IN SIGLA VALORI - S.C. A R. L.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -6072,7 +6286,13 @@
       </c>
       <c r="AF36" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>39,25</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr">
+        <is>
+          <t>+2.1%</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6344,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>94108159.95</t>
+          <t>101603532.22</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -6230,7 +6450,13 @@
       </c>
       <c r="AF37" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>70,73</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>+3.2%</t>
         </is>
       </c>
     </row>
@@ -6384,7 +6610,13 @@
       </c>
       <c r="AF38" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1,69</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr">
+        <is>
+          <t>+0.5%</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6770,13 @@
       </c>
       <c r="AF39" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1,57</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="inlineStr">
+        <is>
+          <t>+0.6%</t>
         </is>
       </c>
     </row>
@@ -6692,7 +6930,13 @@
       </c>
       <c r="AF40" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1,50</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr">
+        <is>
+          <t>+0.5%</t>
         </is>
       </c>
     </row>
@@ -6846,7 +7090,13 @@
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1,44</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr">
+        <is>
+          <t>+0.4%</t>
         </is>
       </c>
     </row>
@@ -7000,7 +7250,13 @@
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>1,93</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>+0.4%</t>
         </is>
       </c>
     </row>
@@ -7062,7 +7318,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -7158,7 +7414,13 @@
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>95,91</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr">
+        <is>
+          <t>+0.4%</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7578,13 @@
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>21,58</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>+3.7%</t>
         </is>
       </c>
     </row>
@@ -7474,7 +7742,13 @@
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>80,70</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>+1.0%</t>
         </is>
       </c>
     </row>
@@ -7632,7 +7906,13 @@
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>2,16</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr">
+        <is>
+          <t>+0.8%</t>
         </is>
       </c>
     </row>
@@ -7674,7 +7954,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>VALORI S.C.A R.L.</t>
+          <t>VALORI S.C.A R.L. - CONSORZIO STABI IN SIGLA VALORI - S.C. A R. L.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -7694,7 +7974,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -7790,7 +8070,13 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>97,17</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>+9.2%</t>
         </is>
       </c>
     </row>
@@ -7837,12 +8123,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>134178919.45</t>
+          <t>137093776.15</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>148353255.91</t>
+          <t>151268112.61</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -7948,7 +8234,13 @@
       </c>
       <c r="AF48" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>12,13</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>+1.4%</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8302,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -8106,7 +8398,113 @@
       </c>
       <c r="AF49" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>90,71</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>+3.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>80128</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sicilia</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>A19</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>A19 PALERMO - CATANIA</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>F77H21007730001</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Lavori di ammodernamento della carreggiata in direzione Catania del viadotto Cannatello, tra i km 84+700 e km 88+920 dell'Autostrada A19 "Palermo - Catania" - Stralcio 1</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Lavori di manutenzione programmata.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>RTI VALORI CONS. STAB. - COSEDIL</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>48692664.4</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>51199397.41</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>191.643</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>A19 0.000–191.643</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>2,47</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>Obra Nueva</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update master state — 2026-06-23 11:50
9 file sincronizzati dalla UI PAVIMOD:
  - data/processed/master_avanzamento.xlsx
  - data/processed/blacklist.json
  - data/cache/opencup_cache.json
  - data/processed/anas_obras_20260415_125514.csv
  - data/processed/anas_obras_20260424_084236.csv
  - data/processed/anas_obras_20260424_122045.csv
  - data/processed/anas_obras_20260616_113605.csv
  - data/processed/anas_obras_20260616_115120.csv
  - data/processed/anas_obras_20260616_131141.csv
</commit_message>
<xml_diff>
--- a/data/processed/master_avanzamento.xlsx
+++ b/data/processed/master_avanzamento.xlsx
@@ -740,7 +740,11 @@
           <t>2,70</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG2" t="inlineStr">
         <is>
           <t>3,53</t>
@@ -904,7 +908,11 @@
           <t>83,14</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG3" t="inlineStr">
         <is>
           <t>84,38</t>
@@ -1068,7 +1076,11 @@
           <t>1,08</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG4" t="inlineStr">
         <is>
           <t>1,87</t>
@@ -1232,7 +1244,11 @@
           <t>39,57</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG5" t="inlineStr">
         <is>
           <t>44,24</t>
@@ -1396,7 +1412,11 @@
           <t>79,71</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG6" t="inlineStr">
         <is>
           <t>83,00</t>
@@ -1560,7 +1580,11 @@
           <t>10,65</t>
         </is>
       </c>
-      <c r="AF7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG7" t="inlineStr">
         <is>
           <t>12,92</t>
@@ -1724,7 +1748,11 @@
           <t>11,95</t>
         </is>
       </c>
-      <c r="AF8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG8" t="inlineStr">
         <is>
           <t>16,63</t>
@@ -1888,7 +1916,11 @@
           <t>95,17</t>
         </is>
       </c>
-      <c r="AF9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">
         <is>
@@ -2048,7 +2080,11 @@
           <t>50,80</t>
         </is>
       </c>
-      <c r="AF10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG10" t="inlineStr">
         <is>
           <t>58,74</t>
@@ -2212,7 +2248,11 @@
           <t>2,52</t>
         </is>
       </c>
-      <c r="AF11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG11" t="inlineStr">
         <is>
           <t>3,12</t>
@@ -2376,7 +2416,11 @@
           <t>25,13</t>
         </is>
       </c>
-      <c r="AF12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG12" t="inlineStr">
         <is>
           <t>27,49</t>
@@ -2540,7 +2584,11 @@
           <t>92,33</t>
         </is>
       </c>
-      <c r="AF13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG13" t="inlineStr">
         <is>
           <t>92,33</t>
@@ -2700,7 +2748,11 @@
           <t>14,90</t>
         </is>
       </c>
-      <c r="AF14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG14" t="inlineStr">
         <is>
           <t>18,51</t>

</xml_diff>

<commit_message>
Update master state — 2026-06-23 12:27
9 file sincronizzati dalla UI PAVIMOD:
  - data/processed/master_avanzamento.xlsx
  - data/processed/blacklist.json
  - data/cache/opencup_cache.json
  - data/processed/anas_obras_20260415_125514.csv
  - data/processed/anas_obras_20260424_084236.csv
  - data/processed/anas_obras_20260424_122045.csv
  - data/processed/anas_obras_20260616_113605.csv
  - data/processed/anas_obras_20260616_115120.csv
  - data/processed/anas_obras_20260616_131141.csv
</commit_message>
<xml_diff>
--- a/data/processed/master_avanzamento.xlsx
+++ b/data/processed/master_avanzamento.xlsx
@@ -2912,7 +2912,11 @@
           <t>3,09</t>
         </is>
       </c>
-      <c r="AF15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG15" t="inlineStr">
         <is>
           <t>5,67</t>
@@ -3072,7 +3076,11 @@
           <t>18,87</t>
         </is>
       </c>
-      <c r="AF16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG16" t="inlineStr">
         <is>
           <t>21,15</t>
@@ -3232,7 +3240,11 @@
           <t>38,05</t>
         </is>
       </c>
-      <c r="AF17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG17" t="inlineStr">
         <is>
           <t>42,02</t>
@@ -3392,7 +3404,11 @@
           <t>3,22</t>
         </is>
       </c>
-      <c r="AF18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG18" t="inlineStr">
         <is>
           <t>3,22</t>
@@ -3552,7 +3568,11 @@
           <t>29,87</t>
         </is>
       </c>
-      <c r="AF19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG19" t="inlineStr">
         <is>
           <t>33,87</t>
@@ -3716,7 +3736,11 @@
           <t>78,03</t>
         </is>
       </c>
-      <c r="AF20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG20" t="inlineStr">
         <is>
           <t>87,37</t>
@@ -3880,7 +3904,11 @@
           <t>98,31</t>
         </is>
       </c>
-      <c r="AF21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG21" t="inlineStr">
         <is>
           <t>99,06</t>
@@ -4040,7 +4068,11 @@
           <t>99,77</t>
         </is>
       </c>
-      <c r="AF22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG22" t="inlineStr">
         <is>
           <t>99,92</t>
@@ -4204,7 +4236,11 @@
           <t>92,07</t>
         </is>
       </c>
-      <c r="AF23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG23" t="inlineStr">
         <is>
           <t>92,47</t>
@@ -4368,7 +4404,11 @@
           <t>96,08</t>
         </is>
       </c>
-      <c r="AF24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG24" t="inlineStr">
         <is>
           <t>96,42</t>
@@ -4532,7 +4572,11 @@
           <t>99,94</t>
         </is>
       </c>
-      <c r="AF25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Non interessa</t>
+        </is>
+      </c>
       <c r="AG25" t="inlineStr">
         <is>
           <t>99,94</t>
@@ -4696,7 +4740,11 @@
           <t>19,13</t>
         </is>
       </c>
-      <c r="AF26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG26" t="inlineStr">
         <is>
           <t>24,48</t>
@@ -4860,7 +4908,11 @@
           <t>7,27</t>
         </is>
       </c>
-      <c r="AF27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG27" t="inlineStr">
         <is>
           <t>7,29</t>
@@ -5024,7 +5076,11 @@
           <t>41,84</t>
         </is>
       </c>
-      <c r="AF28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG28" t="inlineStr">
         <is>
           <t>46,31</t>
@@ -5188,7 +5244,11 @@
           <t>100,00</t>
         </is>
       </c>
-      <c r="AF29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG29" t="inlineStr">
         <is>
           <t>100,00</t>
@@ -5352,7 +5412,11 @@
           <t>89,19</t>
         </is>
       </c>
-      <c r="AF30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG30" t="inlineStr">
         <is>
           <t>92,15</t>
@@ -5516,7 +5580,11 @@
           <t>98,88</t>
         </is>
       </c>
-      <c r="AF31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG31" t="inlineStr">
         <is>
           <t>98,88</t>
@@ -5680,7 +5748,11 @@
           <t>58,95</t>
         </is>
       </c>
-      <c r="AF32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG32" t="inlineStr">
         <is>
           <t>58,95</t>
@@ -5844,7 +5916,11 @@
           <t>60,58</t>
         </is>
       </c>
-      <c r="AF33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG33" t="inlineStr">
         <is>
           <t>62,65</t>
@@ -6008,7 +6084,11 @@
           <t>45,70</t>
         </is>
       </c>
-      <c r="AF34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG34" t="inlineStr">
         <is>
           <t>49,15</t>
@@ -6172,7 +6252,11 @@
           <t>23,77</t>
         </is>
       </c>
-      <c r="AF35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG35" t="inlineStr">
         <is>
           <t>26,23</t>
@@ -6336,7 +6420,11 @@
           <t>37,11</t>
         </is>
       </c>
-      <c r="AF36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG36" t="inlineStr">
         <is>
           <t>39,25</t>
@@ -6500,7 +6588,11 @@
           <t>67,58</t>
         </is>
       </c>
-      <c r="AF37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG37" t="inlineStr">
         <is>
           <t>70,73</t>
@@ -6660,7 +6752,11 @@
           <t>1,20</t>
         </is>
       </c>
-      <c r="AF38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG38" t="inlineStr">
         <is>
           <t>1,69</t>
@@ -6820,7 +6916,11 @@
           <t>0,98</t>
         </is>
       </c>
-      <c r="AF39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG39" t="inlineStr">
         <is>
           <t>1,57</t>
@@ -6980,7 +7080,11 @@
           <t>0,97</t>
         </is>
       </c>
-      <c r="AF40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG40" t="inlineStr">
         <is>
           <t>1,50</t>
@@ -7140,7 +7244,11 @@
           <t>1,02</t>
         </is>
       </c>
-      <c r="AF41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG41" t="inlineStr">
         <is>
           <t>1,44</t>
@@ -7300,7 +7408,11 @@
           <t>1,48</t>
         </is>
       </c>
-      <c r="AF42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG42" t="inlineStr">
         <is>
           <t>1,93</t>
@@ -7464,7 +7576,11 @@
           <t>95,52</t>
         </is>
       </c>
-      <c r="AF43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG43" t="inlineStr">
         <is>
           <t>95,91</t>
@@ -7628,7 +7744,11 @@
           <t>17,86</t>
         </is>
       </c>
-      <c r="AF44" t="inlineStr"/>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG44" t="inlineStr">
         <is>
           <t>21,58</t>
@@ -7792,7 +7912,11 @@
           <t>79,69</t>
         </is>
       </c>
-      <c r="AF45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG45" t="inlineStr">
         <is>
           <t>80,70</t>
@@ -7956,7 +8080,11 @@
           <t>1,33</t>
         </is>
       </c>
-      <c r="AF46" t="inlineStr"/>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG46" t="inlineStr">
         <is>
           <t>2,16</t>
@@ -8120,7 +8248,11 @@
           <t>87,98</t>
         </is>
       </c>
-      <c r="AF47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG47" t="inlineStr">
         <is>
           <t>97,17</t>
@@ -8284,7 +8416,11 @@
           <t>10,69</t>
         </is>
       </c>
-      <c r="AF48" t="inlineStr"/>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG48" t="inlineStr">
         <is>
           <t>12,13</t>
@@ -8448,7 +8584,11 @@
           <t>87,25</t>
         </is>
       </c>
-      <c r="AF49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>In VTiger</t>
+        </is>
+      </c>
       <c r="AG49" t="inlineStr">
         <is>
           <t>90,71</t>
@@ -8588,7 +8728,11 @@
       <c r="AC50" t="inlineStr"/>
       <c r="AD50" t="inlineStr"/>
       <c r="AE50" t="inlineStr"/>
-      <c r="AF50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>Da caricare</t>
+        </is>
+      </c>
       <c r="AG50" t="inlineStr">
         <is>
           <t>2,47</t>

</xml_diff>